<commit_message>
auto: update dashboard report and AI map
</commit_message>
<xml_diff>
--- a/data/typhoon_predictions.xlsx
+++ b/data/typhoon_predictions.xlsx
@@ -489,19 +489,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>48</v>
+        <v>51.6</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>31.9</v>
+        <v>33.3</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="F3" t="n">
-        <v>4.3</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -511,19 +511,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>77.90000000000001</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="C4" t="n">
-        <v>4.8</v>
+        <v>7.2</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>7.3</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="5">
@@ -536,16 +536,16 @@
         <v>100</v>
       </c>
       <c r="C5" t="n">
-        <v>22.8</v>
+        <v>27.6</v>
       </c>
       <c r="D5" t="n">
-        <v>6.7</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>4.1</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="6">
@@ -555,10 +555,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>90.8</v>
+        <v>85.5</v>
       </c>
       <c r="C6" t="n">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -567,7 +567,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>4.4</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="7">
@@ -577,10 +577,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>62.9</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>10.8</v>
+        <v>9.6</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -589,7 +589,7 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="8">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8.699999999999999</v>
+        <v>12.5</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -611,7 +611,7 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>4.5</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="9">
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3.9</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -633,7 +633,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>5.6</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="10">
@@ -655,7 +655,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -665,19 +665,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>10.8</v>
+        <v>4.8</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>2.4</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>5.9</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="12">
@@ -693,13 +693,13 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>3.7</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="13">
@@ -715,13 +715,13 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>1.2</v>
+        <v>4.9</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="14">
@@ -737,13 +737,13 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>4.7</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="15">
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>23.1</v>
+        <v>21.6</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
@@ -765,7 +765,7 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>5.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>10.4</v>
+        <v>15.2</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
@@ -787,7 +787,7 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>6.7</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="17">
@@ -797,19 +797,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>16.8</v>
+        <v>26.4</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>7.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>8.9</v>
+        <v>30.9</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
@@ -831,7 +831,7 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>5.7</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="19">
@@ -841,19 +841,19 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>25.3</v>
+        <v>24</v>
       </c>
       <c r="C19" t="n">
         <v>2.4</v>
       </c>
       <c r="D19" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>7.3</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="20">
@@ -869,13 +869,13 @@
         <v>3.6</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>8</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="21">
@@ -885,13 +885,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>31.6</v>
+        <v>26.3</v>
       </c>
       <c r="C21" t="n">
         <v>2.4</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -919,7 +919,7 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="23">
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>44.5</v>
+        <v>43.2</v>
       </c>
       <c r="C23" t="n">
         <v>0</v>
@@ -941,7 +941,7 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="24">
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>46.3</v>
+        <v>52.4</v>
       </c>
       <c r="C24" t="n">
         <v>0</v>
@@ -963,7 +963,7 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="25">
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>40.7</v>
+        <v>36.7</v>
       </c>
       <c r="C25" t="n">
         <v>0</v>
@@ -985,7 +985,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>6.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="26">
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>33.1</v>
+        <v>29.1</v>
       </c>
       <c r="C26" t="n">
         <v>0</v>
@@ -1007,7 +1007,7 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>6.4</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="27">
@@ -1017,10 +1017,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>57.1</v>
+        <v>51.6</v>
       </c>
       <c r="C27" t="n">
-        <v>3.6</v>
+        <v>2.4</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -1029,7 +1029,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>6.9</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="28">
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>54.5</v>
+        <v>48.1</v>
       </c>
       <c r="C28" t="n">
         <v>0</v>
@@ -1051,7 +1051,7 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>6.9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
@@ -1061,7 +1061,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>26.7</v>
+        <v>32.9</v>
       </c>
       <c r="C29" t="n">
         <v>0</v>
@@ -1073,7 +1073,7 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>7.3</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="30">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>20.8</v>
+        <v>22</v>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -1105,19 +1105,19 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>40.8</v>
+        <v>44.7</v>
       </c>
       <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
         <v>1.2</v>
       </c>
-      <c r="D31" t="n">
-        <v>0</v>
-      </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="32">
@@ -1127,10 +1127,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>43.3</v>
+        <v>36.1</v>
       </c>
       <c r="C32" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
@@ -1139,7 +1139,7 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>7.4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="33">
@@ -1149,10 +1149,10 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="C33" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
@@ -1161,7 +1161,7 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>9.9</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="34">
@@ -1171,19 +1171,19 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>3.6</v>
+        <v>0</v>
       </c>
       <c r="C34" t="n">
         <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>5.2</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="35">
@@ -1193,19 +1193,19 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>30.1</v>
+        <v>19.2</v>
       </c>
       <c r="C35" t="n">
-        <v>3.6</v>
+        <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>6.1</v>
+        <v>15.3</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>9</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="36">
@@ -1215,19 +1215,19 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>28.9</v>
+        <v>14.4</v>
       </c>
       <c r="C36" t="n">
-        <v>3.6</v>
+        <v>0</v>
       </c>
       <c r="D36" t="n">
-        <v>12.7</v>
+        <v>26.5</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>9</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="37">
@@ -1237,19 +1237,19 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>6</v>
+        <v>1.2</v>
       </c>
       <c r="C37" t="n">
         <v>0</v>
       </c>
       <c r="D37" t="n">
-        <v>31.7</v>
+        <v>37.7</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>8.699999999999999</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="38">
@@ -1259,19 +1259,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="C38" t="n">
         <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>36.3</v>
+        <v>52.3</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39">
@@ -1281,19 +1281,19 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>9.6</v>
+        <v>7.2</v>
       </c>
       <c r="C39" t="n">
         <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>54.7</v>
+        <v>64.8</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>7</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="40">
@@ -1303,13 +1303,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>6</v>
+        <v>4.8</v>
       </c>
       <c r="C40" t="n">
         <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>43.3</v>
+        <v>41.9</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
@@ -1325,19 +1325,19 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>4.9</v>
+        <v>2.4</v>
       </c>
       <c r="C41" t="n">
         <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>35.9</v>
+        <v>40.7</v>
       </c>
       <c r="E41" t="n">
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>8.1</v>
+        <v>7.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>